<commit_message>
change human_male to read from audio folder
</commit_message>
<xml_diff>
--- a/corrections/new_entries.xlsx
+++ b/corrections/new_entries.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\wow_vo_webui\corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C940CD65-8D9B-4744-B6DA-4015826BFEF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9911FBCD-D778-4E2E-B86C-023971DA5DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$489</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2782" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3301" uniqueCount="882">
   <si>
     <t>source</t>
   </si>
@@ -2424,6 +2427,422 @@
   </si>
   <si>
     <t>Welcome to the Plaguelands, hero. This is one of the most dangerous frontiers in Azeroth, with the looming threat of the Scourge to our east, and then even further still eastward from there. I am glad to hear that the call of duty and service to the Horde did not fall on deaf ears with you!$B$BIf you are ready to get your hands dirty, then there is plenty for willing and able heroes to do here on the edge of the Plaguelands.</t>
+  </si>
+  <si>
+    <t>Bow in my presence, insect! Surely you can feel the power I hold over you.</t>
+  </si>
+  <si>
+    <t>Niby the Almighty</t>
+  </si>
+  <si>
+    <t>So you have come to Niby to learn the secrets of calling down an infernal servant from the Nether.$B$BSilence! Niby knows all!$B$BNiby is not so quick to part with such knowledge. First, you must assist Niby with a very important task.</t>
+  </si>
+  <si>
+    <t>There is a powerful infernal named Kroshius northeast of this camp. It is why Niby is here. Kroshius is a greater infernal - an infernal that has lasted longer than expected. You see, nub, an infernal crashes down into the earth with great intensity to serve its master but this intensity fades fast. Once the blazing flames have died down, the infernal crumbles.</t>
+  </si>
+  <si>
+    <t>Do not interrupt Niby, fool! I shall rend the flesh from your bones and use your skeletal remains as a coat rack. Now where was I? Oh yes, so, Kroshius lasted nearly ten times longer than any ordinary infernal. I am not sure why but I am confident that with enough study, I could find out.$B$BI need you to recover Kroshius' Infernal Core.</t>
+  </si>
+  <si>
+    <t>If I am to teach you the secrets of summoning an infernal servant, you must destroy Kroshius and bring me the infernal core from his burning remains. This, however, is not as easy as it sounds. Kroshius has all but burned out completely. You must reignite his corpse and raise him from the rubble. To do this, however, you must gather some components from other demonic entities.$B$BMy imp, Impsy, shall set you on your way.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+There was a time when I could ask whatever I wished from those who sought out my master. But now, he takes pretty much anyone in as an apprentice and they can pass through his portals all they please.
+It is upsetting to me, but I do not question his orders. I can only take enjoyment in making fun of the ridiculous clothes you wear or the pathetic look on your face. Even that bores me...
+Even this rambling bores me! Go. Be gone. Share your depressing sense of style with someone else.</t>
+  </si>
+  <si>
+    <t>Sanath Lim-yo</t>
+  </si>
+  <si>
+    <t>Meeting with the Master</t>
+  </si>
+  <si>
+    <t>There was a time when I could ask whatever I wished from those who sought out my master.  But now, you need only ask and I will send you to him.
+It is upsetting to me, but I do not question his orders.  I can only take enjoyment in making fun of the ridiculous clothes you wear or the pathetic look on your face.  Even that bores me...
+Even this rambling bores me!  Do you wish to see my master or not?</t>
+  </si>
+  <si>
+    <t>Magecraft</t>
+  </si>
+  <si>
+    <t>Archmage Xylem awaits your arrival.</t>
+  </si>
+  <si>
+    <t>Salfa</t>
+  </si>
+  <si>
+    <t>Aurora Skycaller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please, leave this place, &lt;name&gt;. You know nothing of what troubles us... </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave me, &lt;race&gt;. You know not what troubles us. </t>
+  </si>
+  <si>
+    <t>Troubled Spirits of Kel'Theril</t>
+  </si>
+  <si>
+    <t>The past of the high elves is something that I do not wish to discuss, &lt;name&gt;. Please, it pains me to think of all that has happened... And that there is no way to make things right.</t>
+  </si>
+  <si>
+    <t>I did not realize ; Forgive my callous words, &lt;class&gt;.
+The mistakes of my ancestors are not what I wish to dwell on, but if your request is truly genuine, then I will help you.
+&lt;Aurora examines the fragments.&gt;
+I believe this is the Crystal of Zin-Malor, an artifact that can contain and control strong arcane forces. It could have been used for good, but the evil intentions of those that stole it caused it to shatter.
+Go to the Temple of Zin-Malor in Azshara - I can only hope the book is still there.</t>
+  </si>
+  <si>
+    <t>The pages have gone untouched for many many years…</t>
+  </si>
+  <si>
+    <t>Fragments of the Past</t>
+  </si>
+  <si>
+    <t>I will be able to help you, if recreating the artifact is truly what you wish to do.
+To seal the pieces back together, I will need items with strong magical qualities. An enchanted thorium bar and five crystal restore... You'll also need to collect some water from what might seem an unlikely place... Find the dire pool along Eldreth Row at Dire Maul in Feralas, and fill this vial.
+While you are gone, I will attempt to glean from these pages the knowledge I need to repair the damage done to the relic.</t>
+  </si>
+  <si>
+    <t>Using these elements, I can fuse the fragments together... to hopefully what they once were.</t>
+  </si>
+  <si>
+    <t>Tormented By the Past</t>
+  </si>
+  <si>
+    <t>I weep for what has happened in the past. Like this crystal, the elves, as a race, have been shattered. I do not know if the pieces will ever again be reunited into one, but my sorrow has been eased by being able to help you with this one small task.
+We must not forget the past, &lt;name&gt;...
+Please take the Crystal of Zin-Malor back to Lake Kel'Theril. You must find a highborne spirit that realizes the error of what was done so long ago. Show the spirit that we have made things right again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We Timbermaw can grant you safe passage through the hold; however, you must prove yourself worthy of our aid. </t>
+  </si>
+  <si>
+    <t>Welcome, adventurer! Are you interested in training in tailoring?</t>
+  </si>
+  <si>
+    <t>Meilosh</t>
+  </si>
+  <si>
+    <t>Do you want to play a game, stinky?</t>
+  </si>
+  <si>
+    <t>If you want the key, you'll have to catch me!</t>
+  </si>
+  <si>
+    <t>I hold the key to lands of free! Catch me and you'll see!</t>
+  </si>
+  <si>
+    <t>Chase me if you dare! I run without a care!</t>
+  </si>
+  <si>
+    <t>Still alive? You do surprise. Watch me as I flee!</t>
+  </si>
+  <si>
+    <t>Why would you ever want to harm me!? Come. Friends we can be!</t>
+  </si>
+  <si>
+    <t>Turn that frown upside down!</t>
+  </si>
+  <si>
+    <t>Die?! You make Pusillin cry!</t>
+  </si>
+  <si>
+    <t>This is the end of the line, no friend of mine!</t>
+  </si>
+  <si>
+    <t>Say hello to my little friends!</t>
+  </si>
+  <si>
+    <t>Pusillin</t>
+  </si>
+  <si>
+    <t>I was sent as a scout to do some damage and gauge the strength of Hearthglen's defenses. Some people in the Alliance feel the little town has more than historical importance. It's not my job to question what that importance is, but regardless, I'm in no shape to continue until I rest up.$B$BIf you're willing, I'd pay handsomely for some help. Start south of here at their camp near the small bulwark they've set up. If you prove strong enough, maybe I could get your help with my main goal.</t>
+  </si>
+  <si>
+    <t>Kirsta Deepshadow</t>
+  </si>
+  <si>
+    <t>Well done, $N. I'm amazed you dealt with them so quickly. Thank you.$B$BI have yet to meet anyone that approves of the Scarlet Crusade and their methods. I believe in the Light as much as anyone else in Stormwind, but they've demonstrated that they only want to kill anyone not loyal to their movement... even innocents.</t>
+  </si>
+  <si>
+    <t>My real mission was to weaken the Scarlet Crusade's outlying forces and then infiltrate Hearthglen to gauge their numbers. I'm still in no shape to do it on my own, so perhaps I could ask you to aid me again, $N? From what information I gathered before being discovered, the Crusade has two important members that are the backbone of their forces outside the town: Huntsman Radley and Cavalier Durgen. Kill them, and we're making progress. They should be along Hearthglen Pass outside the town proper.</t>
+  </si>
+  <si>
+    <t>Thank you, $N. You've been more help than I could have hoped for. The air here just seems to suck my will. I feel tired, and I can tell I'm not getting any better the longer I'm here.$B$BI'm not really sure how I'm going to infiltrate Hearthglen itself and report on how strong the Scarlet Crusade's presence is.$B$BBut that's another matter, before you leave, here, take this... as payment for your help. Thank you again.</t>
+  </si>
+  <si>
+    <t>What? Really? You want to know more? But you've already done so much for me, $N. I couldn't possibly ask you to enter Hearthglen itself on my behalf.$B$BAre you sure, $N? Hearthglen is much more dangerous than the Pass--I cannot provide you any protection  or even information about what you might face.$B$BWell, if you really are willing to help, then enter the town and find a high place to gain a good view of the town. From there you can gauge their numbers and report them back to me. But be careful....</t>
+  </si>
+  <si>
+    <t>You've done it, $N! Thank you!$B$BI'll return to Elling... I mean Stormwind as soon as I can. Here, take this coin, it's the least I can do for you. You're a credit to your people, $N. Thank you and good luck.</t>
+  </si>
+  <si>
+    <t>Demon Dogs</t>
+  </si>
+  <si>
+    <t>If you are going to remain here, I ask only that you earn your keep. We have many nuisances that could use some 'discipline.'$B$BYou can start with the Plaguehounds and their runts.$B$BI cannot offer much in return, but you are guaranteed a warm meal and some conversation should you succeed.</t>
+  </si>
+  <si>
+    <t>Tirion Fordring</t>
+  </si>
+  <si>
+    <t>Well done, $N. Come. Rest. Let us eat and talk of days long past!</t>
+  </si>
+  <si>
+    <t>Blood Tinged Skies</t>
+  </si>
+  <si>
+    <t>Woe to those that foolishly wander into the Plaguelands. All manner of foulness inhabit these woods - from the fanatical Scarlet Crusade, who will kill any that do not bear the mark of the Crusade, to the murderous Scourge, who only look to bolster their numbers by adding more undead to their ranks.$B$BEven the wildlife have been transformed into rapacious, man eating beasts. I ask that you destroy those that would strike from the skies: The Plaguebats.</t>
+  </si>
+  <si>
+    <t>You are a shining example of decency, $r! It has been long since I have felt the blood of heroes pump through my veins. Your acts of bravery are uplifting!</t>
+  </si>
+  <si>
+    <t>Carrion Grubbage</t>
+  </si>
+  <si>
+    <t>My food supplies are running low, $r. I am ashamed to admit that I might not have enough food to share with you.$B$BCould you assist an old man with a simple task? Around here, the only manner of beast unaffected by the ravages of the Plague are the Carrion worms. While rather bland in taste, the meat of the worms can easily be preserved to last for months. I will need several hundred pounds to restock for the coming winter!</t>
+  </si>
+  <si>
+    <t>May the Light watch over you! Bless you, young one.</t>
+  </si>
+  <si>
+    <t>Redemption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You have worked hard, friend. Rest your weary bones and allow me to properly introduce myself.
+</t>
+  </si>
+  <si>
+    <t>The Fordring redemption will be a difficult task. Are you prepared?</t>
+  </si>
+  <si>
+    <t>Of Forgotten Memories</t>
+  </si>
+  <si>
+    <t>To help Taelan regain what he has lost, you must gather items from his past.$B$BThe first such item is a toy that I gave to him on his 7th birthday. It was his most cherished possession: A miniature war hammer; an exact replica of my very own.$B$BAfter I was banished for treason, his mother told him that I had died. He was taken to my false grave at the Undercroft, where he buried the hammer along with my memory - forever.$B$BYou must venture to the Undercroft and recover Taelan's hammer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;Tirion blinks to hold back tears.&gt;$B$BIt was destiny that we meet, $N. You have blessed me with your kindness.
+</t>
+  </si>
+  <si>
+    <t>Of Lost Honor</t>
+  </si>
+  <si>
+    <t>The Order of the Silver Hand was utterly decimated when Uther was slain.$B$BThe boy held out for as long as he could. Pushed to the war torn hamlet of Northdale, he made his final stand.$B$BWere any of the Order left alive, he thought - and did it matter?$B$BIt was with that thought that Taelan threw down the standard of the Order and renounced all that he had known. His honor left upon the blood soaked ground of Northdale.$B$BYou must travel to Northdale and recover that symbol of lost honor.</t>
+  </si>
+  <si>
+    <t>It is as glorious now - even in its tattered state - as the day I looked upon it and took my oath of allegiance.$B$BHis redemption comes and perhaps mine with it...</t>
+  </si>
+  <si>
+    <t>Of Love and Family</t>
+  </si>
+  <si>
+    <t>When Taelan was a child, we would oft visit Caer Darrow on family excursions. On our last visit, an artist by the name of Renfray painted a portrait of us poised along the beachside. It is my fondest memory of both Taelan and Karandra. For it was at that moment, with my wife and son in my arms, that I felt a bond of love and family that I would never know again.$B$BIf this painting still exists, you must find it.$B$BTravel to the ruined island of Caer Darrow and see if the painting or the artist remain.</t>
+  </si>
+  <si>
+    <t>Find Myranda</t>
+  </si>
+  <si>
+    <t>$N, you have done all that I have asked thus far. Only one step remains in your quest of redemption.$B$BYou must deliver the items you have collected to Taelan. Unfortunately, Taelan and his Scarlet Crusaders will attack you on sight.$B$BThere is only one way in which to deliver my message and that is through a guise of deception.$B$BTo the south you will find Uther's tomb. An old and trusted confidant of mine, Myranda, now resides there - seek her out. Show her the items and she will assist you.</t>
+  </si>
+  <si>
+    <t>In Dreams</t>
+  </si>
+  <si>
+    <t>The death of my son at the hands of these monsters will not pass without incident. Take solace in knowing that the Order is reborn.$B$BI now take my place as Highlord of the new Order of the Silver Hand.$B$BThese possessions of my past - they are all that I have to offer for all that you have done. Please, take these as a symbol of my gratitude; all have served me well over the years.$B$BMay we meet again, in better times, and reminisce of days long past... battles hard fought... dreams redeemed.</t>
+  </si>
+  <si>
+    <t>Lord Tirion Fordring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race does not dictate honor, $r. While you remain on my farmstead, I ask that you remember and respect this credo.$B$BI have known orcs who have been as honorable as the most noble of knights and humans who have been as vile as the most ruthless of Scourge.$B$BBut I shall not bore you with tales of my youth! There is much work to be done - if that is what you desire. </t>
+  </si>
+  <si>
+    <t>Sit and listen to my story, $r.</t>
+  </si>
+  <si>
+    <t>I must apologize for not being entirely truthful with you in regards to my identity. I had to be certain that you could be trusted - few people would have selflessly lent assistance to an old and forgotten hermit.$B$BYou have proven yourself as one of those people: A person of integrity and honor.</t>
+  </si>
+  <si>
+    <t>My son, Taelan, was only a child when I was found guilty of treason and banished from the Alliance to live a life in exile. I chose to remain here so that I could watch over him; to somehow insure that he would grow up an honorable man.$B$BAs I had hoped, he took my place as lord of Mardenholde; but in a cruel twist of fate, joined the ranks of the Scarlet Crusade. He is now their Highlord, $r.</t>
+  </si>
+  <si>
+    <t>Indeed. The Scarlet Crusade are an aberration of the Order of the Silver Hand.$B$BYou must believe me, $r; Taelan is a good man. He needs guidance. He needs to remember... remember what it is to be noble and honorable. I know that in his heart, he knows what he does is wrong. Will you help him? Will you help him remember?</t>
+  </si>
+  <si>
+    <t>What Is Going On?</t>
+  </si>
+  <si>
+    <t>This is a chance for the Horde to change the political climate of our war torn world forever. Listen carefully, $N.$B$BFailure of this mission is not an option.</t>
+  </si>
+  <si>
+    <t>The Eastern Kingdoms</t>
+  </si>
+  <si>
+    <t>You bring excellent information, $N.$B$BAs Warchief, it is my duty to do what is best for the Horde. To ensure that the generations that come after us are not forced into a hopeless existence.$B$BThe opportunity to shape our future alliances has fallen into our collective laps. A move to help the dwarves could greatly strengthen our relationships in the Eastern Kingdoms. This, then, is why you must not fail!$B$BAre you prepared?</t>
+  </si>
+  <si>
+    <t>There is no going back beyond this point, $N.</t>
+  </si>
+  <si>
+    <t>The Royal Rescue</t>
+  </si>
+  <si>
+    <t>This strike against the Dark Iron dwarves, if successful, will send a shockwave throughout their entire kingdom.$B$BPrincess Bronzebeard is under the control of Emperor Thaurissan. To free her, you must kill the Emperor. Be warned, your task is doubly dangerous, as Bronzebeard will attack you without question while under the control of the Emperor.$B$BDO NOT HARM HER!</t>
+  </si>
+  <si>
+    <t>The Princess Saved?</t>
+  </si>
+  <si>
+    <t>&lt;Thrall is taken aback by the information you have presented to him.&gt;$B$BA new threat now looms on the horizon. As Magni's years dwindle down, the way shall be opened for this unborn Dark Iron to become ruler of Ironforge.$B$BYou have accomplished what I asked of you and for that, you shall be rewarded.$B$BNow leave me, $N! I must confer with Sylvanas and Cairne.</t>
+  </si>
+  <si>
+    <t>Eitrigg's Wisdom</t>
+  </si>
+  <si>
+    <t>&lt;Thrall appears dismayed by the news you bring.&gt;</t>
+  </si>
+  <si>
+    <t>For The Horde!</t>
+  </si>
+  <si>
+    <t>Rend dares make such grand claims because of the protection he is afforded by the black flight.$B$BYou, $N, will find a way to pass through the Halls of Ascension. You will then find 'Warchief' Rend Blackhand and you will destroy him - FOR THE HORDE!$B$B&lt;Thrall slams a fist down upon his throne.&gt;$B$BThe next time you return to my chambers, you will hold his head high in triumph and then you shall present it to your Warchief. Do this and be honored as a hero of the Horde.</t>
+  </si>
+  <si>
+    <t>You have dealt a crippling blow to the forces of Blackrock, $N. With their Warchief slain, the Blackrock legion is once again thrown into the maw of chaos.$B$BIn honor of your heroics, the people of Kalimdor shall be rewarded!</t>
+  </si>
+  <si>
+    <t>Hidden Enemies</t>
+  </si>
+  <si>
+    <t>One thing I will not tolerate are traitors in our midst, $N. But I would be a fool to play my hand so early--it would not sufficiently cut the corruption out of our lands and only cause the infection to grow worse.$B$BBut you, a young adventurer, could go places my agents could not... could learn the truth... could find the true head of the beast.$B$BIf you are brave enough, then enter Skull Rock to the east of Orgrimmar, find a lieutenant's insignia off one of the Burning Blade there, and return to me.</t>
+  </si>
+  <si>
+    <t>Good, $N! The spirits be praised, perhaps you are the one who will finally put my greatest fears to rest! Who would suspect someone so young and so brave would rise up and champion our cause? You remind me of myself when I was younger. I will ensure that you are justly rewarded for your efforts if we both survive the coming storm.$B$BBut there is time for more praise later. You've not accomplished anything in comparison to what you will face... but this is a good start.</t>
+  </si>
+  <si>
+    <t>Now let us see if this insignia you found is worth the effort.$B$BThere is a warlock within the city who believes he has my trust. He does not know that I realize where his true loyalties lie. He is in fact the leader of the Burning Blade. But do not rush off to do battle with him; he has a purpose, and we shall use him against our enemies.$B$BTake this insignia to him in the Cleft of Shadow here in Orgrimmar, speak to him and see if he believes you are one of his own, then return to me here.</t>
+  </si>
+  <si>
+    <t>Excellent! Most excellent, $c!$B$BWhat you have done this day is only the first step in a much broader foundation--a foundation that we will build the destruction of the Shadow Council on, once and for all.$B$BTell me all he said... and leave not one word out--it may be more important than you realize.</t>
+  </si>
+  <si>
+    <t>Hmm, leaders of the Searing Blade... this concerns me most. If they are the ones of value to Neeru, then those are who we must target first. This satyr... Bazzalan, and the other Neeru mentioned--what was he, a warlock?--must be slain.$B$BReturn to the Cleft of Shadow and enter Ragefire Chasm, $N. Find these two leaders of the Searing Blade, and kill them. But be careful not to let Neeru know it was you who did this. You must retain your identity as one of his $gbrothers:sisters; in arms.</t>
+  </si>
+  <si>
+    <t>I am glad you've returned, $N. Some of those loyal to me brought word immediately that the caverns below Orgrimmar were in disarray now that their leaders have been slain. I even heard reports that Neeru was more than agitated. It seems we've put a dent in his armor. I can't say I'm displeased... even with such a minor victory.</t>
+  </si>
+  <si>
+    <t>I think our next step should be to have you placed close to Neeru. If he is as agitated as reports suggest, then we may accomplish two things. One, you may be able to gain some greater knowledge about the Council or at least the Burning Blade, and two, he may just begin to trust you enough that he asks you to start to aid him. He may very well look at you as someone who can fill the void now that some of the leadership is in turmoil.$B$BReturn to the Cleft and speak to him again, but do not be too overt.</t>
+  </si>
+  <si>
+    <t>Ashenvale? Hmm, I had not heard of any presence of the Council or the Burning Blade in Ashenvale. My spies will investigate, $N. You have done well.$B$BFor now, rest, and keep yourself occupied with other tasks. I will call upon you again soon.$B$BLok-Tar Ogar!</t>
+  </si>
+  <si>
+    <t>What the Wind Carries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is good to see you again, $N. The wind carries with it news from the Eastern Kingdom.$B$BSit, listen. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are you prepared to take on this task?
+</t>
+  </si>
+  <si>
+    <t>The Champion of the Horde</t>
+  </si>
+  <si>
+    <t>I have received word from one of my champions that a way into the lair of the dragon may exist. You are to seek him out.$B$BRexxar wanders the desert wasteland of Desolace, traveling between Stonetalon and Feralas. He awaits your arrival.</t>
+  </si>
+  <si>
+    <t>Victory for the Horde</t>
+  </si>
+  <si>
+    <t>This is a great victory for the Horde, $N. So many times you have honored your Warchief. It is time for the Warchief to honor you.</t>
+  </si>
+  <si>
+    <t>For All To See</t>
+  </si>
+  <si>
+    <t>Overlord Runthak awaits your arrival in the Valley of Strength.$B$B&lt;Thrall salutes you.&gt;$B$BDo not keep your public waiting, hero.</t>
+  </si>
+  <si>
+    <t>The Lord of Blackrock</t>
+  </si>
+  <si>
+    <t>You have honored the Horde once more, $N. The son of Deathwing lays dead. Surely, the evil one stirs.</t>
+  </si>
+  <si>
+    <t>Seek out High Overlord Saurfang in the Valley of Strength.</t>
+  </si>
+  <si>
+    <t>The Brokering of Peace</t>
+  </si>
+  <si>
+    <t>Indeed, this is a most fortuitous turn of events. Were a lasting peace to be made with these creatures, this would certainly give us an advantage in securing Kalimdor from external threats. I will notify the other leaders of the Horde of this immediately, and further diplomats will be dispatched!$B$BAs for you, $N... you have shown courage in both diplomacy and in action. I thank you, as does the entirety of the Horde.</t>
+  </si>
+  <si>
+    <t>All members of the Horde are equal in my eyes, $n. We have all suffered many burdens, and if it were not for wisdom and honor, then we would be no better than the Scourge or my people while our blood was tainted by the demon Mannoroth.$B$BIt is your duty to aid the Horde and to defend our way of life. But it is also your duty to know when quarter and compassion should be given to friend and foe alike.$B$BUnderstand this well. This is the new Horde, not some demon-spawned army who lack freewill.</t>
+  </si>
+  <si>
+    <t>The Shattered Hand has been able to place spies throughout the upper citadel of Blackrock. Though the information gathering process has been slow, we have made discoveries that cannot be ignored.</t>
+  </si>
+  <si>
+    <t>It would appear as if the influence of the Black Dragonflight had extended beyond the borders of the Burning Steppes and into the kingdom of Stormwind itself! The usurper has since been unmasked and ousted.</t>
+  </si>
+  <si>
+    <t>Indeed. The brood mother of the Black Dragonflight had used illusion and trickery to disguise herself as a member of the royal court. Worse yet, she had assumed control of the current Highlord of Stormwind, Bolvar Fordragon.$B$BIt is no wonder that such foolish military decisions had been made. The movement of the Alliance forces as of late had left us scratching our heads. We now understand that the Black Flight was attempting to divide the empire - destroy it from within.</t>
+  </si>
+  <si>
+    <t>&lt;Thrall laughs.&gt;$B$BSo much to learn still, $r.$B$BYou are too young to remember the wars and bloodshed of ages past. Too young to remember the burden of the curse carried by our people.$B$BOur position with the Alliance right now is a tenuous one. Skirmishes and smaller battles do take place, but there is peace - something our people have not known for millennia. Would you give this up and plunge us into the maw of chaos again but against a new foe? One that will not rest until we are all destroyed?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No, $n, you did not. I do not fault you, however, as yours is a mind much like mine was as a youth: Impetuous, rebellious, and often without a single coherent thought! Traits I can no longer afford to express.$B$BEnough lamenting. $R, I have a task for you; one that you may not survive. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;Thrall laughs.&gt;$B$BNoted... Now pay attention, $n. The Black Dragonflight brood mother, Onyxia, has been flushed out from her position of power in Stormwind. She has escaped, fleeing to her lair in Dustwallow Marsh.$B$BShe cannot be allowed to live in such close proximity to our capital cities. We must strike before being struck!$B$BI want her destroyed, $n. </t>
+  </si>
+  <si>
+    <t>Why have you come here, adventurer?</t>
+  </si>
+  <si>
+    <t>Better Late Than Never</t>
+  </si>
+  <si>
+    <t>"The package must be delivered... delivered before I'm trapped here!"$B$BThe cries of a panicked woman feel almost like a whisper floating through the house.  Cowered in the upstairs corner is the apparition of a woman.  She does not seem to be fully cognizant of her surroundings, and she is only vaguely aware of you.$B$B"Are you here to deliver my package?  Please, before it gets much worse!  I was going to ride out of here.  It should still be by my horse... or am I too late?"</t>
+  </si>
+  <si>
+    <t>Janice Felstone</t>
+  </si>
+  <si>
+    <t>A package for an Emma Felstone, you say?  Last known address was Stormwind, four years ago?  Well let me see here...$B$BAccording to what we know, there was an Emma Felstone in the city about four years ago.  Well, I should say possibly - this census I refer to is from five years ago, and I don't have a report of her vacating the city.  This doesn't mean that she is still here though.$B$BWait a second... this package couldn't be for Ol' Emma, could it?</t>
+  </si>
+  <si>
+    <t>Royal Factor Bathrilor</t>
+  </si>
+  <si>
+    <t>A package for a Jeremiah Felstone, with his last known address as Lordaeron... I should be able to assist you.$B$BJeremiah Felstone was in the city before the plague.  Well, I should say the former Jeremiah Felstone - some of the Forsaken have changed their last names to rid themselves of their former countenance.  This case is no exception; the former Jeremiah Felstone is now known as Jeremiah Payson.$B$BWait a minute... isn't he the cockroach vendor?</t>
+  </si>
+  <si>
+    <t>Royal Overseer Bauhaus</t>
+  </si>
+  <si>
+    <t>Tirion nearly collapses when he sees the painting. He begins to sob in an almost frenetic manner.</t>
+  </si>
+  <si>
+    <t>How could I forget? Many of the spirits on this island are cursed to relive their last happy memory before they met their tragic end.$B$BI too am cursed, but not as they - I am one of the few that remembers all...$B$BPerhaps this thing that you ask me is why I haunt these ruins. Perhaps this thing I tell you shall set me free.</t>
+  </si>
+  <si>
+    <t>Artist Renfray</t>
+  </si>
+  <si>
+    <t>The painting... It hung on the wall of my workshop - inside the Order's barracks - for years.$B$BAfter Tirion's trial was over, I knew that I could no longer keep the painting visible. I hid it in a place that they would never think to look.$B$BTravel to Stratholme and make your way deep inside what is now the Scarlet Bastion, search for a painting of our twin moons. Chip away at the paint until you uncover my master work, 'Of Love and Family.'$B$BMay the Light guide your actions.</t>
   </si>
 </sst>
 </file>
@@ -2758,7 +3177,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K472"/>
+  <dimension ref="A1:K564"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
@@ -18954,7 +19373,3030 @@
         <v>-88</v>
       </c>
     </row>
+    <row r="473" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A473" t="s">
+        <v>205</v>
+      </c>
+      <c r="D473" t="s">
+        <v>749</v>
+      </c>
+      <c r="E473">
+        <v>7</v>
+      </c>
+      <c r="F473">
+        <v>0</v>
+      </c>
+      <c r="G473" t="s">
+        <v>750</v>
+      </c>
+      <c r="H473" t="s">
+        <v>12</v>
+      </c>
+      <c r="I473">
+        <v>14469</v>
+      </c>
+      <c r="J473" t="s">
+        <v>749</v>
+      </c>
+      <c r="K473">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="474" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A474" t="s">
+        <v>205</v>
+      </c>
+      <c r="D474" t="s">
+        <v>751</v>
+      </c>
+      <c r="E474">
+        <v>7</v>
+      </c>
+      <c r="F474">
+        <v>0</v>
+      </c>
+      <c r="G474" t="s">
+        <v>750</v>
+      </c>
+      <c r="H474" t="s">
+        <v>12</v>
+      </c>
+      <c r="I474">
+        <v>14469</v>
+      </c>
+      <c r="J474" t="s">
+        <v>751</v>
+      </c>
+      <c r="K474">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="475" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>205</v>
+      </c>
+      <c r="D475" t="s">
+        <v>752</v>
+      </c>
+      <c r="E475">
+        <v>7</v>
+      </c>
+      <c r="F475">
+        <v>0</v>
+      </c>
+      <c r="G475" t="s">
+        <v>750</v>
+      </c>
+      <c r="H475" t="s">
+        <v>12</v>
+      </c>
+      <c r="I475">
+        <v>14469</v>
+      </c>
+      <c r="J475" t="s">
+        <v>752</v>
+      </c>
+      <c r="K475">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="476" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A476" t="s">
+        <v>205</v>
+      </c>
+      <c r="D476" t="s">
+        <v>753</v>
+      </c>
+      <c r="E476">
+        <v>7</v>
+      </c>
+      <c r="F476">
+        <v>0</v>
+      </c>
+      <c r="G476" t="s">
+        <v>750</v>
+      </c>
+      <c r="H476" t="s">
+        <v>12</v>
+      </c>
+      <c r="I476">
+        <v>14469</v>
+      </c>
+      <c r="J476" t="s">
+        <v>753</v>
+      </c>
+      <c r="K476">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A477" t="s">
+        <v>205</v>
+      </c>
+      <c r="D477" t="s">
+        <v>754</v>
+      </c>
+      <c r="E477">
+        <v>7</v>
+      </c>
+      <c r="F477">
+        <v>0</v>
+      </c>
+      <c r="G477" t="s">
+        <v>750</v>
+      </c>
+      <c r="H477" t="s">
+        <v>12</v>
+      </c>
+      <c r="I477">
+        <v>14469</v>
+      </c>
+      <c r="J477" t="s">
+        <v>754</v>
+      </c>
+      <c r="K477">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>205</v>
+      </c>
+      <c r="D478" t="s">
+        <v>755</v>
+      </c>
+      <c r="E478">
+        <v>10</v>
+      </c>
+      <c r="F478">
+        <v>0</v>
+      </c>
+      <c r="G478" t="s">
+        <v>756</v>
+      </c>
+      <c r="H478" t="s">
+        <v>12</v>
+      </c>
+      <c r="I478">
+        <v>8395</v>
+      </c>
+      <c r="J478" t="s">
+        <v>755</v>
+      </c>
+      <c r="K478">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>11</v>
+      </c>
+      <c r="B479">
+        <v>3503</v>
+      </c>
+      <c r="C479" t="s">
+        <v>757</v>
+      </c>
+      <c r="D479" t="s">
+        <v>758</v>
+      </c>
+      <c r="E479">
+        <v>10</v>
+      </c>
+      <c r="F479">
+        <v>0</v>
+      </c>
+      <c r="G479" t="s">
+        <v>756</v>
+      </c>
+      <c r="H479" t="s">
+        <v>12</v>
+      </c>
+      <c r="I479">
+        <v>8395</v>
+      </c>
+      <c r="J479" t="s">
+        <v>755</v>
+      </c>
+      <c r="K479">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>11</v>
+      </c>
+      <c r="B480">
+        <v>8250</v>
+      </c>
+      <c r="C480" t="s">
+        <v>759</v>
+      </c>
+      <c r="D480" t="s">
+        <v>760</v>
+      </c>
+      <c r="E480">
+        <v>10</v>
+      </c>
+      <c r="F480">
+        <v>0</v>
+      </c>
+      <c r="G480" t="s">
+        <v>756</v>
+      </c>
+      <c r="H480" t="s">
+        <v>12</v>
+      </c>
+      <c r="I480">
+        <v>8395</v>
+      </c>
+      <c r="J480" t="s">
+        <v>760</v>
+      </c>
+      <c r="K480">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>205</v>
+      </c>
+      <c r="D481" t="s">
+        <v>774</v>
+      </c>
+      <c r="E481">
+        <v>-77</v>
+      </c>
+      <c r="F481">
+        <v>-77</v>
+      </c>
+      <c r="G481" t="s">
+        <v>761</v>
+      </c>
+      <c r="H481" t="s">
+        <v>12</v>
+      </c>
+      <c r="I481">
+        <v>11556</v>
+      </c>
+      <c r="J481" t="s">
+        <v>774</v>
+      </c>
+      <c r="K481">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>205</v>
+      </c>
+      <c r="D482" t="s">
+        <v>763</v>
+      </c>
+      <c r="E482">
+        <v>10</v>
+      </c>
+      <c r="F482">
+        <v>1</v>
+      </c>
+      <c r="G482" t="s">
+        <v>762</v>
+      </c>
+      <c r="H482" t="s">
+        <v>12</v>
+      </c>
+      <c r="I482">
+        <v>10304</v>
+      </c>
+      <c r="J482" t="s">
+        <v>763</v>
+      </c>
+      <c r="K482">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>205</v>
+      </c>
+      <c r="D483" t="s">
+        <v>764</v>
+      </c>
+      <c r="E483">
+        <v>10</v>
+      </c>
+      <c r="F483">
+        <v>1</v>
+      </c>
+      <c r="G483" t="s">
+        <v>762</v>
+      </c>
+      <c r="H483" t="s">
+        <v>12</v>
+      </c>
+      <c r="I483">
+        <v>10304</v>
+      </c>
+      <c r="J483" t="s">
+        <v>764</v>
+      </c>
+      <c r="K483">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>11</v>
+      </c>
+      <c r="B484">
+        <v>5245</v>
+      </c>
+      <c r="C484" t="s">
+        <v>765</v>
+      </c>
+      <c r="D484" t="s">
+        <v>766</v>
+      </c>
+      <c r="E484">
+        <v>10</v>
+      </c>
+      <c r="F484">
+        <v>1</v>
+      </c>
+      <c r="G484" t="s">
+        <v>762</v>
+      </c>
+      <c r="H484" t="s">
+        <v>12</v>
+      </c>
+      <c r="I484">
+        <v>10304</v>
+      </c>
+      <c r="J484" t="s">
+        <v>765</v>
+      </c>
+      <c r="K484">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>13</v>
+      </c>
+      <c r="B485">
+        <v>5246</v>
+      </c>
+      <c r="C485" t="s">
+        <v>769</v>
+      </c>
+      <c r="D485" t="s">
+        <v>767</v>
+      </c>
+      <c r="E485">
+        <v>10</v>
+      </c>
+      <c r="F485">
+        <v>1</v>
+      </c>
+      <c r="G485" t="s">
+        <v>762</v>
+      </c>
+      <c r="H485" t="s">
+        <v>12</v>
+      </c>
+      <c r="I485">
+        <v>10304</v>
+      </c>
+      <c r="J485" t="s">
+        <v>769</v>
+      </c>
+      <c r="K485">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>11</v>
+      </c>
+      <c r="B486">
+        <v>5246</v>
+      </c>
+      <c r="C486" t="s">
+        <v>769</v>
+      </c>
+      <c r="D486" t="s">
+        <v>768</v>
+      </c>
+      <c r="E486">
+        <v>10</v>
+      </c>
+      <c r="F486">
+        <v>1</v>
+      </c>
+      <c r="G486" t="s">
+        <v>762</v>
+      </c>
+      <c r="H486" t="s">
+        <v>12</v>
+      </c>
+      <c r="I486">
+        <v>10304</v>
+      </c>
+      <c r="J486" t="s">
+        <v>769</v>
+      </c>
+      <c r="K486">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>13</v>
+      </c>
+      <c r="B487">
+        <v>5247</v>
+      </c>
+      <c r="C487" t="s">
+        <v>769</v>
+      </c>
+      <c r="D487" t="s">
+        <v>770</v>
+      </c>
+      <c r="E487">
+        <v>10</v>
+      </c>
+      <c r="F487">
+        <v>1</v>
+      </c>
+      <c r="G487" t="s">
+        <v>762</v>
+      </c>
+      <c r="H487" t="s">
+        <v>12</v>
+      </c>
+      <c r="I487">
+        <v>10304</v>
+      </c>
+      <c r="J487" t="s">
+        <v>769</v>
+      </c>
+      <c r="K487">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="488" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>11</v>
+      </c>
+      <c r="B488">
+        <v>5247</v>
+      </c>
+      <c r="C488" t="s">
+        <v>769</v>
+      </c>
+      <c r="D488" t="s">
+        <v>771</v>
+      </c>
+      <c r="E488">
+        <v>10</v>
+      </c>
+      <c r="F488">
+        <v>1</v>
+      </c>
+      <c r="G488" t="s">
+        <v>762</v>
+      </c>
+      <c r="H488" t="s">
+        <v>12</v>
+      </c>
+      <c r="I488">
+        <v>10304</v>
+      </c>
+      <c r="J488" t="s">
+        <v>769</v>
+      </c>
+      <c r="K488">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>13</v>
+      </c>
+      <c r="B489">
+        <v>5248</v>
+      </c>
+      <c r="C489" t="s">
+        <v>772</v>
+      </c>
+      <c r="D489" t="s">
+        <v>773</v>
+      </c>
+      <c r="E489">
+        <v>10</v>
+      </c>
+      <c r="F489">
+        <v>1</v>
+      </c>
+      <c r="G489" t="s">
+        <v>762</v>
+      </c>
+      <c r="H489" t="s">
+        <v>12</v>
+      </c>
+      <c r="I489">
+        <v>10304</v>
+      </c>
+      <c r="J489" t="s">
+        <v>769</v>
+      </c>
+      <c r="K489">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>205</v>
+      </c>
+      <c r="D490" t="s">
+        <v>775</v>
+      </c>
+      <c r="E490">
+        <v>-77</v>
+      </c>
+      <c r="F490">
+        <v>-77</v>
+      </c>
+      <c r="G490" t="s">
+        <v>776</v>
+      </c>
+      <c r="H490" t="s">
+        <v>12</v>
+      </c>
+      <c r="I490">
+        <v>11557</v>
+      </c>
+      <c r="J490" t="s">
+        <v>775</v>
+      </c>
+      <c r="K490">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>205</v>
+      </c>
+      <c r="D491" t="s">
+        <v>777</v>
+      </c>
+      <c r="E491">
+        <v>-77</v>
+      </c>
+      <c r="F491">
+        <v>-77</v>
+      </c>
+      <c r="G491" t="s">
+        <v>787</v>
+      </c>
+      <c r="H491" t="s">
+        <v>12</v>
+      </c>
+      <c r="I491">
+        <v>14354</v>
+      </c>
+      <c r="J491" t="s">
+        <v>777</v>
+      </c>
+      <c r="K491">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>205</v>
+      </c>
+      <c r="D492" t="s">
+        <v>778</v>
+      </c>
+      <c r="E492">
+        <v>-77</v>
+      </c>
+      <c r="F492">
+        <v>-77</v>
+      </c>
+      <c r="G492" t="s">
+        <v>787</v>
+      </c>
+      <c r="H492" t="s">
+        <v>12</v>
+      </c>
+      <c r="I492">
+        <v>14354</v>
+      </c>
+      <c r="J492" t="s">
+        <v>778</v>
+      </c>
+      <c r="K492">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>205</v>
+      </c>
+      <c r="D493" t="s">
+        <v>779</v>
+      </c>
+      <c r="E493">
+        <v>-77</v>
+      </c>
+      <c r="F493">
+        <v>-77</v>
+      </c>
+      <c r="G493" t="s">
+        <v>787</v>
+      </c>
+      <c r="H493" t="s">
+        <v>12</v>
+      </c>
+      <c r="I493">
+        <v>14354</v>
+      </c>
+      <c r="J493" t="s">
+        <v>779</v>
+      </c>
+      <c r="K493">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="494" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>205</v>
+      </c>
+      <c r="D494" t="s">
+        <v>780</v>
+      </c>
+      <c r="E494">
+        <v>-77</v>
+      </c>
+      <c r="F494">
+        <v>-77</v>
+      </c>
+      <c r="G494" t="s">
+        <v>787</v>
+      </c>
+      <c r="H494" t="s">
+        <v>12</v>
+      </c>
+      <c r="I494">
+        <v>14354</v>
+      </c>
+      <c r="J494" t="s">
+        <v>780</v>
+      </c>
+      <c r="K494">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="495" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A495" t="s">
+        <v>205</v>
+      </c>
+      <c r="D495" t="s">
+        <v>781</v>
+      </c>
+      <c r="E495">
+        <v>-77</v>
+      </c>
+      <c r="F495">
+        <v>-77</v>
+      </c>
+      <c r="G495" t="s">
+        <v>787</v>
+      </c>
+      <c r="H495" t="s">
+        <v>12</v>
+      </c>
+      <c r="I495">
+        <v>14354</v>
+      </c>
+      <c r="J495" t="s">
+        <v>781</v>
+      </c>
+      <c r="K495">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A496" t="s">
+        <v>205</v>
+      </c>
+      <c r="D496" t="s">
+        <v>782</v>
+      </c>
+      <c r="E496">
+        <v>-77</v>
+      </c>
+      <c r="F496">
+        <v>-77</v>
+      </c>
+      <c r="G496" t="s">
+        <v>787</v>
+      </c>
+      <c r="H496" t="s">
+        <v>12</v>
+      </c>
+      <c r="I496">
+        <v>14354</v>
+      </c>
+      <c r="J496" t="s">
+        <v>782</v>
+      </c>
+      <c r="K496">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="497" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A497" t="s">
+        <v>205</v>
+      </c>
+      <c r="D497" t="s">
+        <v>783</v>
+      </c>
+      <c r="E497">
+        <v>-77</v>
+      </c>
+      <c r="F497">
+        <v>-77</v>
+      </c>
+      <c r="G497" t="s">
+        <v>787</v>
+      </c>
+      <c r="H497" t="s">
+        <v>12</v>
+      </c>
+      <c r="I497">
+        <v>14354</v>
+      </c>
+      <c r="J497" t="s">
+        <v>783</v>
+      </c>
+      <c r="K497">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="498" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A498" t="s">
+        <v>205</v>
+      </c>
+      <c r="D498" t="s">
+        <v>784</v>
+      </c>
+      <c r="E498">
+        <v>-77</v>
+      </c>
+      <c r="F498">
+        <v>-77</v>
+      </c>
+      <c r="G498" t="s">
+        <v>787</v>
+      </c>
+      <c r="H498" t="s">
+        <v>12</v>
+      </c>
+      <c r="I498">
+        <v>14354</v>
+      </c>
+      <c r="J498" t="s">
+        <v>784</v>
+      </c>
+      <c r="K498">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A499" t="s">
+        <v>205</v>
+      </c>
+      <c r="D499" t="s">
+        <v>785</v>
+      </c>
+      <c r="E499">
+        <v>-77</v>
+      </c>
+      <c r="F499">
+        <v>-77</v>
+      </c>
+      <c r="G499" t="s">
+        <v>787</v>
+      </c>
+      <c r="H499" t="s">
+        <v>12</v>
+      </c>
+      <c r="I499">
+        <v>14354</v>
+      </c>
+      <c r="J499" t="s">
+        <v>785</v>
+      </c>
+      <c r="K499">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="500" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A500" t="s">
+        <v>205</v>
+      </c>
+      <c r="D500" t="s">
+        <v>786</v>
+      </c>
+      <c r="E500">
+        <v>-77</v>
+      </c>
+      <c r="F500">
+        <v>-77</v>
+      </c>
+      <c r="G500" t="s">
+        <v>787</v>
+      </c>
+      <c r="H500" t="s">
+        <v>12</v>
+      </c>
+      <c r="I500">
+        <v>14354</v>
+      </c>
+      <c r="J500" t="s">
+        <v>786</v>
+      </c>
+      <c r="K500">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="501" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A501" t="s">
+        <v>13</v>
+      </c>
+      <c r="B501">
+        <v>6004</v>
+      </c>
+      <c r="C501" t="s">
+        <v>222</v>
+      </c>
+      <c r="D501" t="s">
+        <v>788</v>
+      </c>
+      <c r="E501">
+        <v>1</v>
+      </c>
+      <c r="F501">
+        <v>1</v>
+      </c>
+      <c r="G501" t="s">
+        <v>789</v>
+      </c>
+      <c r="H501" t="s">
+        <v>12</v>
+      </c>
+      <c r="I501">
+        <v>11610</v>
+      </c>
+      <c r="J501" t="s">
+        <v>788</v>
+      </c>
+      <c r="K501">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="502" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A502" t="s">
+        <v>11</v>
+      </c>
+      <c r="B502">
+        <v>6004</v>
+      </c>
+      <c r="C502" t="s">
+        <v>222</v>
+      </c>
+      <c r="D502" t="s">
+        <v>790</v>
+      </c>
+      <c r="E502">
+        <v>1</v>
+      </c>
+      <c r="F502">
+        <v>1</v>
+      </c>
+      <c r="G502" t="s">
+        <v>789</v>
+      </c>
+      <c r="H502" t="s">
+        <v>12</v>
+      </c>
+      <c r="I502">
+        <v>11610</v>
+      </c>
+      <c r="J502" t="s">
+        <v>790</v>
+      </c>
+      <c r="K502">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="503" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A503" t="s">
+        <v>13</v>
+      </c>
+      <c r="B503">
+        <v>6023</v>
+      </c>
+      <c r="C503" t="s">
+        <v>222</v>
+      </c>
+      <c r="D503" t="s">
+        <v>791</v>
+      </c>
+      <c r="E503">
+        <v>1</v>
+      </c>
+      <c r="F503">
+        <v>1</v>
+      </c>
+      <c r="G503" t="s">
+        <v>789</v>
+      </c>
+      <c r="H503" t="s">
+        <v>12</v>
+      </c>
+      <c r="I503">
+        <v>11610</v>
+      </c>
+      <c r="J503" t="s">
+        <v>791</v>
+      </c>
+      <c r="K503">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="504" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A504" t="s">
+        <v>11</v>
+      </c>
+      <c r="B504">
+        <v>6023</v>
+      </c>
+      <c r="C504" t="s">
+        <v>222</v>
+      </c>
+      <c r="D504" t="s">
+        <v>792</v>
+      </c>
+      <c r="E504">
+        <v>1</v>
+      </c>
+      <c r="F504">
+        <v>1</v>
+      </c>
+      <c r="G504" t="s">
+        <v>789</v>
+      </c>
+      <c r="H504" t="s">
+        <v>12</v>
+      </c>
+      <c r="I504">
+        <v>11610</v>
+      </c>
+      <c r="J504" t="s">
+        <v>792</v>
+      </c>
+      <c r="K504">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="505" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A505" t="s">
+        <v>13</v>
+      </c>
+      <c r="B505">
+        <v>6025</v>
+      </c>
+      <c r="C505" t="s">
+        <v>222</v>
+      </c>
+      <c r="D505" t="s">
+        <v>793</v>
+      </c>
+      <c r="E505">
+        <v>1</v>
+      </c>
+      <c r="F505">
+        <v>1</v>
+      </c>
+      <c r="G505" t="s">
+        <v>789</v>
+      </c>
+      <c r="H505" t="s">
+        <v>12</v>
+      </c>
+      <c r="I505">
+        <v>11610</v>
+      </c>
+      <c r="J505" t="s">
+        <v>793</v>
+      </c>
+      <c r="K505">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="506" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A506" t="s">
+        <v>11</v>
+      </c>
+      <c r="B506">
+        <v>6025</v>
+      </c>
+      <c r="C506" t="s">
+        <v>222</v>
+      </c>
+      <c r="D506" t="s">
+        <v>794</v>
+      </c>
+      <c r="E506">
+        <v>1</v>
+      </c>
+      <c r="F506">
+        <v>1</v>
+      </c>
+      <c r="G506" t="s">
+        <v>789</v>
+      </c>
+      <c r="H506" t="s">
+        <v>12</v>
+      </c>
+      <c r="I506">
+        <v>11610</v>
+      </c>
+      <c r="J506" t="s">
+        <v>794</v>
+      </c>
+      <c r="K506">
+        <v>-88</v>
+      </c>
+    </row>
+    <row r="507" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A507" t="s">
+        <v>13</v>
+      </c>
+      <c r="B507">
+        <v>5542</v>
+      </c>
+      <c r="C507" t="s">
+        <v>795</v>
+      </c>
+      <c r="D507" t="s">
+        <v>796</v>
+      </c>
+      <c r="E507">
+        <v>1</v>
+      </c>
+      <c r="F507">
+        <v>0</v>
+      </c>
+      <c r="G507" t="s">
+        <v>797</v>
+      </c>
+      <c r="H507" t="s">
+        <v>12</v>
+      </c>
+      <c r="I507">
+        <v>1855</v>
+      </c>
+      <c r="J507" t="s">
+        <v>796</v>
+      </c>
+      <c r="K507">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A508" t="s">
+        <v>11</v>
+      </c>
+      <c r="B508">
+        <v>5542</v>
+      </c>
+      <c r="C508" t="s">
+        <v>795</v>
+      </c>
+      <c r="D508" t="s">
+        <v>798</v>
+      </c>
+      <c r="E508">
+        <v>1</v>
+      </c>
+      <c r="F508">
+        <v>0</v>
+      </c>
+      <c r="G508" t="s">
+        <v>797</v>
+      </c>
+      <c r="H508" t="s">
+        <v>12</v>
+      </c>
+      <c r="I508">
+        <v>1855</v>
+      </c>
+      <c r="J508" t="s">
+        <v>798</v>
+      </c>
+      <c r="K508">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A509" t="s">
+        <v>13</v>
+      </c>
+      <c r="B509">
+        <v>5543</v>
+      </c>
+      <c r="C509" t="s">
+        <v>799</v>
+      </c>
+      <c r="D509" t="s">
+        <v>800</v>
+      </c>
+      <c r="E509">
+        <v>1</v>
+      </c>
+      <c r="F509">
+        <v>0</v>
+      </c>
+      <c r="G509" t="s">
+        <v>797</v>
+      </c>
+      <c r="H509" t="s">
+        <v>12</v>
+      </c>
+      <c r="I509">
+        <v>1855</v>
+      </c>
+      <c r="J509" t="s">
+        <v>800</v>
+      </c>
+      <c r="K509">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A510" t="s">
+        <v>11</v>
+      </c>
+      <c r="B510">
+        <v>5543</v>
+      </c>
+      <c r="C510" t="s">
+        <v>799</v>
+      </c>
+      <c r="D510" t="s">
+        <v>801</v>
+      </c>
+      <c r="E510">
+        <v>1</v>
+      </c>
+      <c r="F510">
+        <v>0</v>
+      </c>
+      <c r="G510" t="s">
+        <v>797</v>
+      </c>
+      <c r="H510" t="s">
+        <v>12</v>
+      </c>
+      <c r="I510">
+        <v>1855</v>
+      </c>
+      <c r="J510" t="s">
+        <v>801</v>
+      </c>
+      <c r="K510">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A511" t="s">
+        <v>13</v>
+      </c>
+      <c r="B511">
+        <v>5544</v>
+      </c>
+      <c r="C511" t="s">
+        <v>802</v>
+      </c>
+      <c r="D511" t="s">
+        <v>803</v>
+      </c>
+      <c r="E511">
+        <v>1</v>
+      </c>
+      <c r="F511">
+        <v>0</v>
+      </c>
+      <c r="G511" t="s">
+        <v>797</v>
+      </c>
+      <c r="H511" t="s">
+        <v>12</v>
+      </c>
+      <c r="I511">
+        <v>1855</v>
+      </c>
+      <c r="J511" t="s">
+        <v>803</v>
+      </c>
+      <c r="K511">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="512" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A512" t="s">
+        <v>11</v>
+      </c>
+      <c r="B512">
+        <v>5544</v>
+      </c>
+      <c r="C512" t="s">
+        <v>802</v>
+      </c>
+      <c r="D512" t="s">
+        <v>804</v>
+      </c>
+      <c r="E512">
+        <v>1</v>
+      </c>
+      <c r="F512">
+        <v>0</v>
+      </c>
+      <c r="G512" t="s">
+        <v>797</v>
+      </c>
+      <c r="H512" t="s">
+        <v>12</v>
+      </c>
+      <c r="I512">
+        <v>1855</v>
+      </c>
+      <c r="J512" t="s">
+        <v>804</v>
+      </c>
+      <c r="K512">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A513" t="s">
+        <v>13</v>
+      </c>
+      <c r="B513">
+        <v>5742</v>
+      </c>
+      <c r="C513" t="s">
+        <v>805</v>
+      </c>
+      <c r="D513" t="s">
+        <v>806</v>
+      </c>
+      <c r="E513">
+        <v>1</v>
+      </c>
+      <c r="F513">
+        <v>0</v>
+      </c>
+      <c r="G513" t="s">
+        <v>797</v>
+      </c>
+      <c r="H513" t="s">
+        <v>12</v>
+      </c>
+      <c r="I513">
+        <v>1855</v>
+      </c>
+      <c r="J513" t="s">
+        <v>806</v>
+      </c>
+      <c r="K513">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="514" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A514" t="s">
+        <v>11</v>
+      </c>
+      <c r="B514">
+        <v>5742</v>
+      </c>
+      <c r="C514" t="s">
+        <v>805</v>
+      </c>
+      <c r="D514" t="s">
+        <v>807</v>
+      </c>
+      <c r="E514">
+        <v>1</v>
+      </c>
+      <c r="F514">
+        <v>0</v>
+      </c>
+      <c r="G514" t="s">
+        <v>797</v>
+      </c>
+      <c r="H514" t="s">
+        <v>12</v>
+      </c>
+      <c r="I514">
+        <v>1855</v>
+      </c>
+      <c r="J514" t="s">
+        <v>807</v>
+      </c>
+      <c r="K514">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A515" t="s">
+        <v>13</v>
+      </c>
+      <c r="B515">
+        <v>5781</v>
+      </c>
+      <c r="C515" t="s">
+        <v>808</v>
+      </c>
+      <c r="D515" t="s">
+        <v>809</v>
+      </c>
+      <c r="E515">
+        <v>1</v>
+      </c>
+      <c r="F515">
+        <v>0</v>
+      </c>
+      <c r="G515" t="s">
+        <v>797</v>
+      </c>
+      <c r="H515" t="s">
+        <v>12</v>
+      </c>
+      <c r="I515">
+        <v>1855</v>
+      </c>
+      <c r="J515" t="s">
+        <v>809</v>
+      </c>
+      <c r="K515">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="516" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A516" t="s">
+        <v>11</v>
+      </c>
+      <c r="B516">
+        <v>5781</v>
+      </c>
+      <c r="C516" t="s">
+        <v>808</v>
+      </c>
+      <c r="D516" t="s">
+        <v>810</v>
+      </c>
+      <c r="E516">
+        <v>1</v>
+      </c>
+      <c r="F516">
+        <v>0</v>
+      </c>
+      <c r="G516" t="s">
+        <v>797</v>
+      </c>
+      <c r="H516" t="s">
+        <v>12</v>
+      </c>
+      <c r="I516">
+        <v>1855</v>
+      </c>
+      <c r="J516" t="s">
+        <v>810</v>
+      </c>
+      <c r="K516">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="517" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A517" t="s">
+        <v>13</v>
+      </c>
+      <c r="B517">
+        <v>5845</v>
+      </c>
+      <c r="C517" t="s">
+        <v>811</v>
+      </c>
+      <c r="D517" t="s">
+        <v>812</v>
+      </c>
+      <c r="E517">
+        <v>1</v>
+      </c>
+      <c r="F517">
+        <v>0</v>
+      </c>
+      <c r="G517" t="s">
+        <v>797</v>
+      </c>
+      <c r="H517" t="s">
+        <v>12</v>
+      </c>
+      <c r="I517">
+        <v>1855</v>
+      </c>
+      <c r="J517" t="s">
+        <v>812</v>
+      </c>
+      <c r="K517">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="518" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A518" t="s">
+        <v>11</v>
+      </c>
+      <c r="B518">
+        <v>5845</v>
+      </c>
+      <c r="C518" t="s">
+        <v>811</v>
+      </c>
+      <c r="D518" t="s">
+        <v>813</v>
+      </c>
+      <c r="E518">
+        <v>1</v>
+      </c>
+      <c r="F518">
+        <v>0</v>
+      </c>
+      <c r="G518" t="s">
+        <v>797</v>
+      </c>
+      <c r="H518" t="s">
+        <v>12</v>
+      </c>
+      <c r="I518">
+        <v>1855</v>
+      </c>
+      <c r="J518" t="s">
+        <v>813</v>
+      </c>
+      <c r="K518">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="519" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A519" t="s">
+        <v>13</v>
+      </c>
+      <c r="B519">
+        <v>5846</v>
+      </c>
+      <c r="C519" t="s">
+        <v>814</v>
+      </c>
+      <c r="D519" t="s">
+        <v>815</v>
+      </c>
+      <c r="E519">
+        <v>1</v>
+      </c>
+      <c r="F519">
+        <v>0</v>
+      </c>
+      <c r="G519" t="s">
+        <v>797</v>
+      </c>
+      <c r="H519" t="s">
+        <v>12</v>
+      </c>
+      <c r="I519">
+        <v>1855</v>
+      </c>
+      <c r="J519" t="s">
+        <v>815</v>
+      </c>
+      <c r="K519">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="520" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A520" t="s">
+        <v>11</v>
+      </c>
+      <c r="B520">
+        <v>5848</v>
+      </c>
+      <c r="C520" t="s">
+        <v>814</v>
+      </c>
+      <c r="D520" t="s">
+        <v>878</v>
+      </c>
+      <c r="E520">
+        <v>1</v>
+      </c>
+      <c r="F520">
+        <v>0</v>
+      </c>
+      <c r="G520" t="s">
+        <v>797</v>
+      </c>
+      <c r="H520" t="s">
+        <v>12</v>
+      </c>
+      <c r="I520">
+        <v>1855</v>
+      </c>
+      <c r="J520" t="s">
+        <v>878</v>
+      </c>
+      <c r="K520">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="521" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A521" t="s">
+        <v>13</v>
+      </c>
+      <c r="B521">
+        <v>5861</v>
+      </c>
+      <c r="C521" t="s">
+        <v>816</v>
+      </c>
+      <c r="D521" t="s">
+        <v>817</v>
+      </c>
+      <c r="E521">
+        <v>1</v>
+      </c>
+      <c r="F521">
+        <v>0</v>
+      </c>
+      <c r="G521" t="s">
+        <v>797</v>
+      </c>
+      <c r="H521" t="s">
+        <v>12</v>
+      </c>
+      <c r="I521">
+        <v>1855</v>
+      </c>
+      <c r="J521" t="s">
+        <v>817</v>
+      </c>
+      <c r="K521">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A522" t="s">
+        <v>11</v>
+      </c>
+      <c r="B522">
+        <v>5944</v>
+      </c>
+      <c r="C522" t="s">
+        <v>818</v>
+      </c>
+      <c r="D522" t="s">
+        <v>819</v>
+      </c>
+      <c r="E522">
+        <v>1</v>
+      </c>
+      <c r="F522">
+        <v>0</v>
+      </c>
+      <c r="G522" t="s">
+        <v>820</v>
+      </c>
+      <c r="H522" t="s">
+        <v>12</v>
+      </c>
+      <c r="I522">
+        <v>12126</v>
+      </c>
+      <c r="J522" t="s">
+        <v>819</v>
+      </c>
+      <c r="K522">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A523" t="s">
+        <v>205</v>
+      </c>
+      <c r="D523" t="s">
+        <v>821</v>
+      </c>
+      <c r="E523">
+        <v>1</v>
+      </c>
+      <c r="F523">
+        <v>0</v>
+      </c>
+      <c r="G523" t="s">
+        <v>797</v>
+      </c>
+      <c r="H523" t="s">
+        <v>12</v>
+      </c>
+      <c r="I523">
+        <v>1855</v>
+      </c>
+      <c r="J523" t="s">
+        <v>821</v>
+      </c>
+      <c r="K523">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A524" t="s">
+        <v>205</v>
+      </c>
+      <c r="D524" t="s">
+        <v>822</v>
+      </c>
+      <c r="E524">
+        <v>1</v>
+      </c>
+      <c r="F524">
+        <v>0</v>
+      </c>
+      <c r="G524" t="s">
+        <v>797</v>
+      </c>
+      <c r="H524" t="s">
+        <v>12</v>
+      </c>
+      <c r="I524">
+        <v>1855</v>
+      </c>
+      <c r="J524" t="s">
+        <v>822</v>
+      </c>
+      <c r="K524">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A525" t="s">
+        <v>205</v>
+      </c>
+      <c r="D525" t="s">
+        <v>823</v>
+      </c>
+      <c r="E525">
+        <v>1</v>
+      </c>
+      <c r="F525">
+        <v>0</v>
+      </c>
+      <c r="G525" t="s">
+        <v>797</v>
+      </c>
+      <c r="H525" t="s">
+        <v>12</v>
+      </c>
+      <c r="I525">
+        <v>1855</v>
+      </c>
+      <c r="J525" t="s">
+        <v>823</v>
+      </c>
+      <c r="K525">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="526" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A526" t="s">
+        <v>205</v>
+      </c>
+      <c r="D526" t="s">
+        <v>824</v>
+      </c>
+      <c r="E526">
+        <v>1</v>
+      </c>
+      <c r="F526">
+        <v>0</v>
+      </c>
+      <c r="G526" t="s">
+        <v>797</v>
+      </c>
+      <c r="H526" t="s">
+        <v>12</v>
+      </c>
+      <c r="I526">
+        <v>1855</v>
+      </c>
+      <c r="J526" t="s">
+        <v>824</v>
+      </c>
+      <c r="K526">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A527" t="s">
+        <v>205</v>
+      </c>
+      <c r="D527" t="s">
+        <v>825</v>
+      </c>
+      <c r="E527">
+        <v>1</v>
+      </c>
+      <c r="F527">
+        <v>0</v>
+      </c>
+      <c r="G527" t="s">
+        <v>797</v>
+      </c>
+      <c r="H527" t="s">
+        <v>12</v>
+      </c>
+      <c r="I527">
+        <v>1855</v>
+      </c>
+      <c r="J527" t="s">
+        <v>825</v>
+      </c>
+      <c r="K527">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A528" t="s">
+        <v>11</v>
+      </c>
+      <c r="B528">
+        <v>4001</v>
+      </c>
+      <c r="C528" t="s">
+        <v>826</v>
+      </c>
+      <c r="D528" t="s">
+        <v>827</v>
+      </c>
+      <c r="E528">
+        <v>2</v>
+      </c>
+      <c r="F528">
+        <v>0</v>
+      </c>
+      <c r="G528" t="s">
+        <v>387</v>
+      </c>
+      <c r="H528" t="s">
+        <v>12</v>
+      </c>
+      <c r="I528">
+        <v>4949</v>
+      </c>
+      <c r="J528" t="s">
+        <v>827</v>
+      </c>
+      <c r="K528">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A529" t="s">
+        <v>13</v>
+      </c>
+      <c r="B529">
+        <v>4002</v>
+      </c>
+      <c r="C529" t="s">
+        <v>828</v>
+      </c>
+      <c r="D529" t="s">
+        <v>829</v>
+      </c>
+      <c r="E529">
+        <v>2</v>
+      </c>
+      <c r="F529">
+        <v>0</v>
+      </c>
+      <c r="G529" t="s">
+        <v>387</v>
+      </c>
+      <c r="H529" t="s">
+        <v>12</v>
+      </c>
+      <c r="I529">
+        <v>4949</v>
+      </c>
+      <c r="J529" t="s">
+        <v>829</v>
+      </c>
+      <c r="K529">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="530" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A530" t="s">
+        <v>11</v>
+      </c>
+      <c r="B530">
+        <v>4002</v>
+      </c>
+      <c r="C530" t="s">
+        <v>828</v>
+      </c>
+      <c r="D530" t="s">
+        <v>830</v>
+      </c>
+      <c r="E530">
+        <v>2</v>
+      </c>
+      <c r="F530">
+        <v>0</v>
+      </c>
+      <c r="G530" t="s">
+        <v>387</v>
+      </c>
+      <c r="H530" t="s">
+        <v>12</v>
+      </c>
+      <c r="I530">
+        <v>4949</v>
+      </c>
+      <c r="J530" t="s">
+        <v>830</v>
+      </c>
+      <c r="K530">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A531" t="s">
+        <v>13</v>
+      </c>
+      <c r="B531">
+        <v>4003</v>
+      </c>
+      <c r="C531" t="s">
+        <v>831</v>
+      </c>
+      <c r="D531" t="s">
+        <v>832</v>
+      </c>
+      <c r="E531">
+        <v>2</v>
+      </c>
+      <c r="F531">
+        <v>0</v>
+      </c>
+      <c r="G531" t="s">
+        <v>387</v>
+      </c>
+      <c r="H531" t="s">
+        <v>12</v>
+      </c>
+      <c r="I531">
+        <v>4949</v>
+      </c>
+      <c r="J531" t="s">
+        <v>832</v>
+      </c>
+      <c r="K531">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="532" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A532" t="s">
+        <v>11</v>
+      </c>
+      <c r="B532">
+        <v>4004</v>
+      </c>
+      <c r="C532" t="s">
+        <v>833</v>
+      </c>
+      <c r="D532" t="s">
+        <v>834</v>
+      </c>
+      <c r="E532">
+        <v>2</v>
+      </c>
+      <c r="F532">
+        <v>0</v>
+      </c>
+      <c r="G532" t="s">
+        <v>387</v>
+      </c>
+      <c r="H532" t="s">
+        <v>12</v>
+      </c>
+      <c r="I532">
+        <v>4949</v>
+      </c>
+      <c r="J532" t="s">
+        <v>834</v>
+      </c>
+      <c r="K532">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A533" t="s">
+        <v>11</v>
+      </c>
+      <c r="B533">
+        <v>4941</v>
+      </c>
+      <c r="C533" t="s">
+        <v>835</v>
+      </c>
+      <c r="D533" t="s">
+        <v>836</v>
+      </c>
+      <c r="E533">
+        <v>2</v>
+      </c>
+      <c r="F533">
+        <v>0</v>
+      </c>
+      <c r="G533" t="s">
+        <v>387</v>
+      </c>
+      <c r="H533" t="s">
+        <v>12</v>
+      </c>
+      <c r="I533">
+        <v>4949</v>
+      </c>
+      <c r="J533" t="s">
+        <v>836</v>
+      </c>
+      <c r="K533">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="534" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A534" t="s">
+        <v>13</v>
+      </c>
+      <c r="B534">
+        <v>4974</v>
+      </c>
+      <c r="C534" t="s">
+        <v>837</v>
+      </c>
+      <c r="D534" t="s">
+        <v>838</v>
+      </c>
+      <c r="E534">
+        <v>2</v>
+      </c>
+      <c r="F534">
+        <v>0</v>
+      </c>
+      <c r="G534" t="s">
+        <v>387</v>
+      </c>
+      <c r="H534" t="s">
+        <v>12</v>
+      </c>
+      <c r="I534">
+        <v>4949</v>
+      </c>
+      <c r="J534" t="s">
+        <v>838</v>
+      </c>
+      <c r="K534">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="535" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A535" t="s">
+        <v>11</v>
+      </c>
+      <c r="B535">
+        <v>4974</v>
+      </c>
+      <c r="C535" t="s">
+        <v>837</v>
+      </c>
+      <c r="D535" t="s">
+        <v>839</v>
+      </c>
+      <c r="E535">
+        <v>2</v>
+      </c>
+      <c r="F535">
+        <v>0</v>
+      </c>
+      <c r="G535" t="s">
+        <v>387</v>
+      </c>
+      <c r="H535" t="s">
+        <v>12</v>
+      </c>
+      <c r="I535">
+        <v>4949</v>
+      </c>
+      <c r="J535" t="s">
+        <v>839</v>
+      </c>
+      <c r="K535">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A536" t="s">
+        <v>13</v>
+      </c>
+      <c r="B536">
+        <v>5726</v>
+      </c>
+      <c r="C536" t="s">
+        <v>840</v>
+      </c>
+      <c r="D536" t="s">
+        <v>841</v>
+      </c>
+      <c r="E536">
+        <v>2</v>
+      </c>
+      <c r="F536">
+        <v>0</v>
+      </c>
+      <c r="G536" t="s">
+        <v>387</v>
+      </c>
+      <c r="H536" t="s">
+        <v>12</v>
+      </c>
+      <c r="I536">
+        <v>4949</v>
+      </c>
+      <c r="J536" t="s">
+        <v>841</v>
+      </c>
+      <c r="K536">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A537" t="s">
+        <v>11</v>
+      </c>
+      <c r="B537">
+        <v>5726</v>
+      </c>
+      <c r="C537" t="s">
+        <v>840</v>
+      </c>
+      <c r="D537" t="s">
+        <v>842</v>
+      </c>
+      <c r="E537">
+        <v>2</v>
+      </c>
+      <c r="F537">
+        <v>0</v>
+      </c>
+      <c r="G537" t="s">
+        <v>387</v>
+      </c>
+      <c r="H537" t="s">
+        <v>12</v>
+      </c>
+      <c r="I537">
+        <v>4949</v>
+      </c>
+      <c r="J537" t="s">
+        <v>842</v>
+      </c>
+      <c r="K537">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A538" t="s">
+        <v>13</v>
+      </c>
+      <c r="B538">
+        <v>5727</v>
+      </c>
+      <c r="C538" t="s">
+        <v>840</v>
+      </c>
+      <c r="D538" t="s">
+        <v>843</v>
+      </c>
+      <c r="E538">
+        <v>2</v>
+      </c>
+      <c r="F538">
+        <v>0</v>
+      </c>
+      <c r="G538" t="s">
+        <v>387</v>
+      </c>
+      <c r="H538" t="s">
+        <v>12</v>
+      </c>
+      <c r="I538">
+        <v>4949</v>
+      </c>
+      <c r="J538" t="s">
+        <v>843</v>
+      </c>
+      <c r="K538">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="539" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A539" t="s">
+        <v>11</v>
+      </c>
+      <c r="B539">
+        <v>5727</v>
+      </c>
+      <c r="C539" t="s">
+        <v>840</v>
+      </c>
+      <c r="D539" t="s">
+        <v>844</v>
+      </c>
+      <c r="E539">
+        <v>2</v>
+      </c>
+      <c r="F539">
+        <v>0</v>
+      </c>
+      <c r="G539" t="s">
+        <v>387</v>
+      </c>
+      <c r="H539" t="s">
+        <v>12</v>
+      </c>
+      <c r="I539">
+        <v>4949</v>
+      </c>
+      <c r="J539" t="s">
+        <v>844</v>
+      </c>
+      <c r="K539">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A540" t="s">
+        <v>13</v>
+      </c>
+      <c r="B540">
+        <v>5728</v>
+      </c>
+      <c r="C540" t="s">
+        <v>840</v>
+      </c>
+      <c r="D540" t="s">
+        <v>845</v>
+      </c>
+      <c r="E540">
+        <v>2</v>
+      </c>
+      <c r="F540">
+        <v>0</v>
+      </c>
+      <c r="G540" t="s">
+        <v>387</v>
+      </c>
+      <c r="H540" t="s">
+        <v>12</v>
+      </c>
+      <c r="I540">
+        <v>4949</v>
+      </c>
+      <c r="J540" t="s">
+        <v>845</v>
+      </c>
+      <c r="K540">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A541" t="s">
+        <v>11</v>
+      </c>
+      <c r="B541">
+        <v>5728</v>
+      </c>
+      <c r="C541" t="s">
+        <v>840</v>
+      </c>
+      <c r="D541" t="s">
+        <v>846</v>
+      </c>
+      <c r="E541">
+        <v>2</v>
+      </c>
+      <c r="F541">
+        <v>0</v>
+      </c>
+      <c r="G541" t="s">
+        <v>387</v>
+      </c>
+      <c r="H541" t="s">
+        <v>12</v>
+      </c>
+      <c r="I541">
+        <v>4949</v>
+      </c>
+      <c r="J541" t="s">
+        <v>846</v>
+      </c>
+      <c r="K541">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="542" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A542" t="s">
+        <v>13</v>
+      </c>
+      <c r="B542">
+        <v>5729</v>
+      </c>
+      <c r="C542" t="s">
+        <v>840</v>
+      </c>
+      <c r="D542" t="s">
+        <v>847</v>
+      </c>
+      <c r="E542">
+        <v>2</v>
+      </c>
+      <c r="F542">
+        <v>0</v>
+      </c>
+      <c r="G542" t="s">
+        <v>387</v>
+      </c>
+      <c r="H542" t="s">
+        <v>12</v>
+      </c>
+      <c r="I542">
+        <v>4949</v>
+      </c>
+      <c r="J542" t="s">
+        <v>847</v>
+      </c>
+      <c r="K542">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="543" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A543" t="s">
+        <v>11</v>
+      </c>
+      <c r="B543">
+        <v>5730</v>
+      </c>
+      <c r="C543" t="s">
+        <v>840</v>
+      </c>
+      <c r="D543" t="s">
+        <v>848</v>
+      </c>
+      <c r="E543">
+        <v>2</v>
+      </c>
+      <c r="F543">
+        <v>0</v>
+      </c>
+      <c r="G543" t="s">
+        <v>387</v>
+      </c>
+      <c r="H543" t="s">
+        <v>12</v>
+      </c>
+      <c r="I543">
+        <v>4949</v>
+      </c>
+      <c r="J543" t="s">
+        <v>848</v>
+      </c>
+      <c r="K543">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A544" t="s">
+        <v>13</v>
+      </c>
+      <c r="B544">
+        <v>6566</v>
+      </c>
+      <c r="C544" t="s">
+        <v>849</v>
+      </c>
+      <c r="D544" t="s">
+        <v>850</v>
+      </c>
+      <c r="E544">
+        <v>2</v>
+      </c>
+      <c r="F544">
+        <v>0</v>
+      </c>
+      <c r="G544" t="s">
+        <v>387</v>
+      </c>
+      <c r="H544" t="s">
+        <v>12</v>
+      </c>
+      <c r="I544">
+        <v>4949</v>
+      </c>
+      <c r="J544" t="s">
+        <v>850</v>
+      </c>
+      <c r="K544">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="545" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A545" t="s">
+        <v>11</v>
+      </c>
+      <c r="B545">
+        <v>6566</v>
+      </c>
+      <c r="C545" t="s">
+        <v>849</v>
+      </c>
+      <c r="D545" t="s">
+        <v>851</v>
+      </c>
+      <c r="E545">
+        <v>2</v>
+      </c>
+      <c r="F545">
+        <v>0</v>
+      </c>
+      <c r="G545" t="s">
+        <v>387</v>
+      </c>
+      <c r="H545" t="s">
+        <v>12</v>
+      </c>
+      <c r="I545">
+        <v>4949</v>
+      </c>
+      <c r="J545" t="s">
+        <v>851</v>
+      </c>
+      <c r="K545">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A546" t="s">
+        <v>13</v>
+      </c>
+      <c r="B546">
+        <v>6567</v>
+      </c>
+      <c r="C546" t="s">
+        <v>852</v>
+      </c>
+      <c r="D546" t="s">
+        <v>853</v>
+      </c>
+      <c r="E546">
+        <v>2</v>
+      </c>
+      <c r="F546">
+        <v>0</v>
+      </c>
+      <c r="G546" t="s">
+        <v>387</v>
+      </c>
+      <c r="H546" t="s">
+        <v>12</v>
+      </c>
+      <c r="I546">
+        <v>4949</v>
+      </c>
+      <c r="J546" t="s">
+        <v>853</v>
+      </c>
+      <c r="K546">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A547" t="s">
+        <v>11</v>
+      </c>
+      <c r="B547">
+        <v>7490</v>
+      </c>
+      <c r="C547" t="s">
+        <v>854</v>
+      </c>
+      <c r="D547" t="s">
+        <v>855</v>
+      </c>
+      <c r="E547">
+        <v>2</v>
+      </c>
+      <c r="F547">
+        <v>0</v>
+      </c>
+      <c r="G547" t="s">
+        <v>387</v>
+      </c>
+      <c r="H547" t="s">
+        <v>12</v>
+      </c>
+      <c r="I547">
+        <v>4949</v>
+      </c>
+      <c r="J547" t="s">
+        <v>855</v>
+      </c>
+      <c r="K547">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A548" t="s">
+        <v>13</v>
+      </c>
+      <c r="B548">
+        <v>7491</v>
+      </c>
+      <c r="C548" t="s">
+        <v>856</v>
+      </c>
+      <c r="D548" t="s">
+        <v>857</v>
+      </c>
+      <c r="E548">
+        <v>2</v>
+      </c>
+      <c r="F548">
+        <v>0</v>
+      </c>
+      <c r="G548" t="s">
+        <v>387</v>
+      </c>
+      <c r="H548" t="s">
+        <v>12</v>
+      </c>
+      <c r="I548">
+        <v>4949</v>
+      </c>
+      <c r="J548" t="s">
+        <v>857</v>
+      </c>
+      <c r="K548">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A549" t="s">
+        <v>11</v>
+      </c>
+      <c r="B549">
+        <v>7783</v>
+      </c>
+      <c r="C549" t="s">
+        <v>858</v>
+      </c>
+      <c r="D549" t="s">
+        <v>859</v>
+      </c>
+      <c r="E549">
+        <v>2</v>
+      </c>
+      <c r="F549">
+        <v>0</v>
+      </c>
+      <c r="G549" t="s">
+        <v>387</v>
+      </c>
+      <c r="H549" t="s">
+        <v>12</v>
+      </c>
+      <c r="I549">
+        <v>4949</v>
+      </c>
+      <c r="J549" t="s">
+        <v>859</v>
+      </c>
+      <c r="K549">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A550" t="s">
+        <v>13</v>
+      </c>
+      <c r="B550">
+        <v>7784</v>
+      </c>
+      <c r="C550" t="s">
+        <v>858</v>
+      </c>
+      <c r="D550" t="s">
+        <v>860</v>
+      </c>
+      <c r="E550">
+        <v>2</v>
+      </c>
+      <c r="F550">
+        <v>0</v>
+      </c>
+      <c r="G550" t="s">
+        <v>387</v>
+      </c>
+      <c r="H550" t="s">
+        <v>12</v>
+      </c>
+      <c r="I550">
+        <v>4949</v>
+      </c>
+      <c r="J550" t="s">
+        <v>860</v>
+      </c>
+      <c r="K550">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A551" t="s">
+        <v>11</v>
+      </c>
+      <c r="B551">
+        <v>8485</v>
+      </c>
+      <c r="C551" t="s">
+        <v>861</v>
+      </c>
+      <c r="D551" t="s">
+        <v>862</v>
+      </c>
+      <c r="E551">
+        <v>2</v>
+      </c>
+      <c r="F551">
+        <v>0</v>
+      </c>
+      <c r="G551" t="s">
+        <v>387</v>
+      </c>
+      <c r="H551" t="s">
+        <v>12</v>
+      </c>
+      <c r="I551">
+        <v>4949</v>
+      </c>
+      <c r="J551" t="s">
+        <v>862</v>
+      </c>
+      <c r="K551">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A552" t="s">
+        <v>205</v>
+      </c>
+      <c r="D552" t="s">
+        <v>863</v>
+      </c>
+      <c r="E552">
+        <v>2</v>
+      </c>
+      <c r="F552">
+        <v>0</v>
+      </c>
+      <c r="G552" t="s">
+        <v>387</v>
+      </c>
+      <c r="H552" t="s">
+        <v>12</v>
+      </c>
+      <c r="I552">
+        <v>4949</v>
+      </c>
+      <c r="J552" t="s">
+        <v>863</v>
+      </c>
+      <c r="K552">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="553" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A553" t="s">
+        <v>205</v>
+      </c>
+      <c r="D553" t="s">
+        <v>864</v>
+      </c>
+      <c r="E553">
+        <v>2</v>
+      </c>
+      <c r="F553">
+        <v>0</v>
+      </c>
+      <c r="G553" t="s">
+        <v>387</v>
+      </c>
+      <c r="H553" t="s">
+        <v>12</v>
+      </c>
+      <c r="I553">
+        <v>4949</v>
+      </c>
+      <c r="J553" t="s">
+        <v>864</v>
+      </c>
+      <c r="K553">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="554" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A554" t="s">
+        <v>205</v>
+      </c>
+      <c r="D554" t="s">
+        <v>865</v>
+      </c>
+      <c r="E554">
+        <v>2</v>
+      </c>
+      <c r="F554">
+        <v>0</v>
+      </c>
+      <c r="G554" t="s">
+        <v>387</v>
+      </c>
+      <c r="H554" t="s">
+        <v>12</v>
+      </c>
+      <c r="I554">
+        <v>4949</v>
+      </c>
+      <c r="J554" t="s">
+        <v>865</v>
+      </c>
+      <c r="K554">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="555" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A555" t="s">
+        <v>205</v>
+      </c>
+      <c r="D555" t="s">
+        <v>866</v>
+      </c>
+      <c r="E555">
+        <v>2</v>
+      </c>
+      <c r="F555">
+        <v>0</v>
+      </c>
+      <c r="G555" t="s">
+        <v>387</v>
+      </c>
+      <c r="H555" t="s">
+        <v>12</v>
+      </c>
+      <c r="I555">
+        <v>4949</v>
+      </c>
+      <c r="J555" t="s">
+        <v>866</v>
+      </c>
+      <c r="K555">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="556" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A556" t="s">
+        <v>205</v>
+      </c>
+      <c r="D556" t="s">
+        <v>867</v>
+      </c>
+      <c r="E556">
+        <v>2</v>
+      </c>
+      <c r="F556">
+        <v>0</v>
+      </c>
+      <c r="G556" t="s">
+        <v>387</v>
+      </c>
+      <c r="H556" t="s">
+        <v>12</v>
+      </c>
+      <c r="I556">
+        <v>4949</v>
+      </c>
+      <c r="J556" t="s">
+        <v>867</v>
+      </c>
+      <c r="K556">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="557" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A557" t="s">
+        <v>205</v>
+      </c>
+      <c r="D557" t="s">
+        <v>868</v>
+      </c>
+      <c r="E557">
+        <v>2</v>
+      </c>
+      <c r="F557">
+        <v>0</v>
+      </c>
+      <c r="G557" t="s">
+        <v>387</v>
+      </c>
+      <c r="H557" t="s">
+        <v>12</v>
+      </c>
+      <c r="I557">
+        <v>4949</v>
+      </c>
+      <c r="J557" t="s">
+        <v>868</v>
+      </c>
+      <c r="K557">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="558" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A558" t="s">
+        <v>205</v>
+      </c>
+      <c r="D558" t="s">
+        <v>869</v>
+      </c>
+      <c r="E558">
+        <v>2</v>
+      </c>
+      <c r="F558">
+        <v>0</v>
+      </c>
+      <c r="G558" t="s">
+        <v>387</v>
+      </c>
+      <c r="H558" t="s">
+        <v>12</v>
+      </c>
+      <c r="I558">
+        <v>4949</v>
+      </c>
+      <c r="J558" t="s">
+        <v>869</v>
+      </c>
+      <c r="K558">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="559" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A559" t="s">
+        <v>205</v>
+      </c>
+      <c r="D559" t="s">
+        <v>870</v>
+      </c>
+      <c r="E559">
+        <v>10</v>
+      </c>
+      <c r="F559">
+        <v>1</v>
+      </c>
+      <c r="G559" t="s">
+        <v>762</v>
+      </c>
+      <c r="H559" t="s">
+        <v>12</v>
+      </c>
+      <c r="I559">
+        <v>10304</v>
+      </c>
+      <c r="J559" t="s">
+        <v>870</v>
+      </c>
+      <c r="K559">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="560" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A560" t="s">
+        <v>13</v>
+      </c>
+      <c r="B560">
+        <v>5021</v>
+      </c>
+      <c r="C560" t="s">
+        <v>871</v>
+      </c>
+      <c r="D560" t="s">
+        <v>872</v>
+      </c>
+      <c r="E560">
+        <v>1</v>
+      </c>
+      <c r="F560">
+        <v>1</v>
+      </c>
+      <c r="G560" t="s">
+        <v>873</v>
+      </c>
+      <c r="H560" t="s">
+        <v>12</v>
+      </c>
+      <c r="I560">
+        <v>10778</v>
+      </c>
+      <c r="J560" t="s">
+        <v>872</v>
+      </c>
+      <c r="K560">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="561" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A561" t="s">
+        <v>11</v>
+      </c>
+      <c r="B561">
+        <v>5022</v>
+      </c>
+      <c r="C561" t="s">
+        <v>871</v>
+      </c>
+      <c r="D561" t="s">
+        <v>874</v>
+      </c>
+      <c r="E561">
+        <v>1</v>
+      </c>
+      <c r="F561">
+        <v>0</v>
+      </c>
+      <c r="G561" t="s">
+        <v>875</v>
+      </c>
+      <c r="H561" t="s">
+        <v>12</v>
+      </c>
+      <c r="I561">
+        <v>10782</v>
+      </c>
+      <c r="J561" t="s">
+        <v>874</v>
+      </c>
+      <c r="K561">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="562" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A562" t="s">
+        <v>11</v>
+      </c>
+      <c r="B562">
+        <v>5023</v>
+      </c>
+      <c r="C562" t="s">
+        <v>871</v>
+      </c>
+      <c r="D562" t="s">
+        <v>876</v>
+      </c>
+      <c r="E562">
+        <v>5</v>
+      </c>
+      <c r="F562">
+        <v>0</v>
+      </c>
+      <c r="G562" t="s">
+        <v>877</v>
+      </c>
+      <c r="H562" t="s">
+        <v>12</v>
+      </c>
+      <c r="I562">
+        <v>10781</v>
+      </c>
+      <c r="J562" t="s">
+        <v>876</v>
+      </c>
+      <c r="K562">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="563" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A563" t="s">
+        <v>11</v>
+      </c>
+      <c r="B563">
+        <v>5846</v>
+      </c>
+      <c r="C563" t="s">
+        <v>814</v>
+      </c>
+      <c r="D563" t="s">
+        <v>879</v>
+      </c>
+      <c r="E563">
+        <v>1</v>
+      </c>
+      <c r="F563">
+        <v>1</v>
+      </c>
+      <c r="G563" t="s">
+        <v>880</v>
+      </c>
+      <c r="H563" t="s">
+        <v>12</v>
+      </c>
+      <c r="I563">
+        <v>11936</v>
+      </c>
+      <c r="J563" t="s">
+        <v>879</v>
+      </c>
+      <c r="K563">
+        <v>-77</v>
+      </c>
+    </row>
+    <row r="564" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A564" t="s">
+        <v>13</v>
+      </c>
+      <c r="B564">
+        <v>5848</v>
+      </c>
+      <c r="C564" t="s">
+        <v>814</v>
+      </c>
+      <c r="D564" t="s">
+        <v>881</v>
+      </c>
+      <c r="E564">
+        <v>1</v>
+      </c>
+      <c r="F564">
+        <v>1</v>
+      </c>
+      <c r="G564" t="s">
+        <v>880</v>
+      </c>
+      <c r="H564" t="s">
+        <v>12</v>
+      </c>
+      <c r="I564">
+        <v>11936</v>
+      </c>
+      <c r="J564" t="s">
+        <v>881</v>
+      </c>
+      <c r="K564">
+        <v>-77</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K489" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="J467:J469">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>